<commit_message>
Show rebates in the demo
The sample telecom sheet now has a rebate column (리베이트(번호이동)).
The AI maps it like any other column, the rule parser reads the values,
and September's confirmed rebates are loaded for comparison.

A rebate is a settlement amount, so a changed rebate is never promoted
automatically: scene 4 marks it as needing human approval even when no
anomaly rule fires, and scene 6 shows the reviewer approving the
350,000 -> 400,000 change. Scene 7 adds a fourth question that looks up
rebates that went up; the "calculate settlement" refusal moves to q4.

Recordings made before this change no longer match, so rehearse again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLKdkKWPUzyGX5JHxp1CmB
</commit_message>
<xml_diff>
--- a/demo/moduon-ai-demo/data/a_telecom_price_2610.xlsx
+++ b/demo/moduon-ai-demo/data/a_telecom_price_2610.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -433,6 +433,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,6 +491,11 @@
           <t>비고</t>
         </is>
       </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>리베이트(번호이동)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -517,6 +523,9 @@
       <c r="G5" t="n">
         <v>300000</v>
       </c>
+      <c r="I5" t="n">
+        <v>300000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -544,6 +553,9 @@
       <c r="G6" t="n">
         <v>300000</v>
       </c>
+      <c r="I6" t="n">
+        <v>300000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -571,6 +583,9 @@
       <c r="G7" t="n">
         <v>350000</v>
       </c>
+      <c r="I7" t="n">
+        <v>400000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -603,6 +618,9 @@
           <t>번호이동 지원금 조정(10/1부)</t>
         </is>
       </c>
+      <c r="I8" t="n">
+        <v>250000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -634,6 +652,9 @@
         <is>
           <t>신규 출시</t>
         </is>
+      </c>
+      <c r="I9" t="n">
+        <v>450000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>